<commit_message>
Enhance onboarding flow security and functionality
- Implemented RBAC and SQL sanitization for Master Portal KPI execution
- Upgraded Setup Wizard secret_vault to use Standard KMS (boto3)
- Implemented rate limiting for Setup Wizard submission
- Parameterized TDS effective date in Setup Wizard and DB schema
- Secured Agreement print route with login_required and Markdown parsing
- Updated conversation.xlsx with security recommendations
- Added NEWS.xlsx with requested webapp prompts
</commit_message>
<xml_diff>
--- a/conversation.xlsx
+++ b/conversation.xlsx
@@ -1,109 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
-  <si>
-    <t>Category</t>
-  </si>
-  <si>
-    <t>Information</t>
-  </si>
-  <si>
-    <t>Society Details</t>
-  </si>
-  <si>
-    <t>Administrator</t>
-  </si>
-  <si>
-    <t>Instructions</t>
-  </si>
-  <si>
-    <t>Society Compliance</t>
-  </si>
-  <si>
-    <t>TAN &amp; TDS Rates</t>
-  </si>
-  <si>
-    <t>GSTIN &amp; GST Rate</t>
-  </si>
-  <si>
-    <t>Apartment Charges</t>
-  </si>
-  <si>
-    <t>Vendor Charges</t>
-  </si>
-  <si>
-    <t>Accounts</t>
-  </si>
-  <si>
-    <t>Brought Forward</t>
-  </si>
-  <si>
-    <t>Agreement</t>
-  </si>
-  <si>
-    <t>Let's start with the basics — your society's name, address, and contact details. This only takes a minute, and you can always update it later from Settings.</t>
-  </si>
-  <si>
-    <t>This is where you set your SIGNING_SECRET, the key that keeps every QR gate-pass for your society safe. Pick something strong, write it down somewhere safe, and don't worry — you won't need to touch this again unless you ever reissue codes.</t>
-  </si>
-  <si>
-    <t>New here? This page walks you through what EstateHub does and how the portals fit together. Skim it now, or come back to it anytime from the README link.</t>
-  </si>
-  <si>
-    <t>A few one-time decisions about how your society handles GST, TDS, and fund calculations. If you're not sure, the pre-filled defaults are sensible for most societies — you (or your accountant) can always revisit these later.</t>
-  </si>
-  <si>
-    <t>These rates are pre-filled with the current statutory defaults, so most societies can simply confirm and move on. Only change a rate if your accountant has told you it's different for your society.</t>
-  </si>
-  <si>
-    <t>If your society is registered for GST, enter your GSTIN here. The turnover and exemption limits below are set by Master and apply to every society, so they're shown for reference only.</t>
-  </si>
-  <si>
-    <t>Set the default maintenance amount, due date, and fund rates that will apply to every apartment. Don't worry — you can still set special charges for individual flats later if you need to.</t>
-  </si>
-  <si>
-    <t>Quickly set your standard vendor pass rates for 1-day, 7-day, and 1-month passes. These apply society-wide and can be adjusted anytime from the Admin portal.</t>
-  </si>
-  <si>
-    <t>This is where your society's Chart of Accounts lives, already set up and ready to use. You just need to add your accounting start date and, if you have one, your payment QR code.</t>
-  </si>
-  <si>
-    <t>If your society is moving from another system or a manual register, enter the opening balances here so your books start off accurate. If you're starting fresh, feel free to leave these at zero and skip ahead.</t>
-  </si>
-  <si>
-    <t>Almost done! Please read through the terms, then type 'I AGREE' and enter your password to finish setup. Once you're in, you'll be able to bulk-enroll your apartments, owners, vendors, and security staff right away.</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -122,13 +47,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -416,107 +408,125 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Risk Level</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Finding</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Recommendation</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>13</v>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Master Portal</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>KPI Inspector allows raw SQL execution without strict RBAC or query sanitization.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Implement RBAC, SQL-sanitization. Add confirmation for DELETE/DROP by requiring 'DELETE THIS SOCIETY'.</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>14</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Setup Wizard</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SIGNING_SECRET uses reversible encryption. Vault key compromise exposes secrets.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Use Standard KMS to handle encryption/decryption of the QR secret.</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Setup Wizard</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>No rate limiting on submission. Hardcoded TDS effective date to 2024-04-01.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Enforce rate limiting. Parameterize TDS effective date (prompt for Date).</t>
+        </is>
       </c>
     </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2">
-      <c r="A11" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2">
-      <c r="A12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" t="s">
-        <v>23</v>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Agreement Print</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Unauthenticated access to /print_doc/agreement. Raw markdown rendered instead of HTML.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Add @login_required check. Convert Markdown to HTML before escaping.</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
6 statements and jurisdiction awreness
</commit_message>
<xml_diff>
--- a/conversation.xlsx
+++ b/conversation.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -640,19 +640,19 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>Society Details</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>State / Jurisdiction</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Select the society's state accurately. It decides inter-state (IGST) vs intra-state (CGST+SGST) tax on RCM vendor payments, and which state's statutory Balance Sheet head-mapping and Sinking/Repair Fund rate defaults apply (jurisdiction-aware rules are fully live for Uttar Pradesh; other states use generic/Union-law figures until their own regime is added).</t>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>EstateHub is jurisdiction-aware: select the society's state accurately. It decides inter-state (IGST) vs intra-state (CGST+SGST) tax on RCM vendor payments, and which state's statutory Balance Sheet head-mapping and Sinking/Repair Fund rate defaults apply (jurisdiction-aware rules are fully live for Uttar Pradesh; other states use generic/Union-law figures until their own regime is added).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
aoa bye_laws audit fixes
</commit_message>
<xml_diff>
--- a/conversation.xlsx
+++ b/conversation.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20.03" customWidth="1" style="1" min="1" max="1"/>
@@ -656,6 +656,23 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Bye-Laws Adoption</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Provisional until a resolution</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Tick what your Association has actually adopted from the Model Bye-Laws 2011. Nothing here changes how dues, voting or NOC work until a General Body resolution (2/3) is recorded and linked by Master. Clauses the engine enforces (bye-laws 7, 39, 46, 49) can be varied but not dropped. Leave a clause alone if you have not discussed it — it follows the Model Bye-Laws as written.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Phase 2 part 3: resolution/minutes/poll signing, ratification and rule-application registers, compliance certificate, statute verification, undivided-interest fill, refreshed wizard guidance
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019qaZTLaGEuMoCXJKb6KUif
</commit_message>
<xml_diff>
--- a/conversation.xlsx
+++ b/conversation.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20.03" customWidth="1" style="2" min="1" max="1"/>
@@ -473,211 +473,260 @@
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="3">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Society Operations</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Society Duty Hours</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Select the appropriate security duty hours: 8 hours (three shifts a day) or 12 hours (day and night shifts). This sets the shift pattern for the security roster.</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Instructions</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Before you start</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Keep ready: the society's registration details, the list of flats with owners' emails and mobile numbers, TAN and GSTIN (if any), last year's closing balances, and your advocate's and CA's contact details. Nothing is final until you confirm on the Review step.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Society Details</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>State / Jurisdiction</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>EstateHub is jurisdiction-aware: select the society's state accurately. It decides inter-state (IGST) vs intra-state (CGST+SGST) tax on RCM vendor payments, and which state's statutory Balance Sheet head-mapping and Sinking/Repair Fund rate defaults apply (jurisdiction-aware rules are fully live for Uttar Pradesh; other states use generic/Union-law figures until their own regime is added).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="3">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Administrator</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Security Shifts</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Ensure your Signing Secret is kept highly secure. Set Gate Logic appropriately based on whether you use the App, QR Code, or Both for entry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="3">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Society Compliance</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>KPI Link Rules</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Review the KPI_link_rules for relevant Indian statutory compliance laws. Keep GST and TDS rules up to date according to the latest acts and bye-laws.</t>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Step-up password and office-bearers</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Enter the Secretary's name, phone, email and signature image: they print on notices, NOCs and agreements. Create your step-up password and keep it safe: it only confirms sensitive actions (re-issuing QR codes, key rotation); the server creates and guards the society's signing keys itself. The Managing Committee (President, Secretary, Treasurer and others) is appointed after your flats and logins exist, under Settings &gt; Society governance &gt; Managing Committee; each post needs a flat, name, email, phone and signature image, or it shows as incomplete. Set Gate Logic (App, QR Code or Both) and the security duty hours (8 hours, three shifts, or 12 hours, day and night) for the security roster.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="3">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Legal Regime Selection</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Your state's rules</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Pick the state whose Act, Rules and Model Bye-Laws govern your society. Rows marked unverified have not yet been confirmed by your Treasurer or Auditor against the source text; they are shown for reference and do not drive any enforcement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="3">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Funds</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Which funds you keep</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Tick the funds your society actually keeps. A fund the state prescribes is required; any other fund is your society's choice by General Body resolution. Rates and opening balances are entered later.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1" s="3">
+      <c r="A7" t="inlineStr">
         <is>
           <t>TAN &amp; TDS Rates</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>TDS Rates</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Fetch the latest TDS Rates as prescribed by the Indian Income Tax Act. The effective date defaults to 1 April of the current financial year; change it only if the rates apply from another date.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="3">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="8" ht="15" customHeight="1" s="3">
+      <c r="A8" t="inlineStr">
         <is>
           <t>GSTIN &amp; GST Rate</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>GST Rates &amp; Settings</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Check your state's GST thresholds. Ensure you enter the correct GSTIN if your turnover exceeds the exemption limit.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="3">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="9" ht="15" customHeight="1" s="3">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>State Act &amp; Rules</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Compliance</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Review the statutory rules and the links to the Acts and Rules that apply to your society. Keep GST and TDS rules up to date with the latest notifications. Anything marked provisional or unverified appears on your compliance certificate as an exception until it is confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="3">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Model Bye-Laws Adoption</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Provisional until a resolution</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Tick what your Association has actually adopted from the Model Bye-Laws 2011. Nothing here changes how dues, voting or NOC work until a General Body resolution (2/3) is recorded by your society admin under Settings &gt; Society governance; it then activates automatically. Clauses the engine enforces (bye-laws 7, 39, 46, 49) can be varied but not dropped. Leave a clause alone if you have not discussed it — it follows the Model Bye-Laws as written.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="3">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Apartment Charges</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Apartment Fines &amp; Charges</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Configure Apartment maintenance charges and fines based on the society's bye-laws (e.g., per sq ft vs fixed). Set realistic due dates and interest rates.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="3">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="12" ht="15" customHeight="1" s="3">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Vendor Charges</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Vendor Fines &amp; Charges</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Set vendor penalties for late work or non-compliance (1-day, 7-day, 1-month). Ensure these match the vendor contracts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="3">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Accounts</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Vendor passes</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Set the price of Vendor Passes (1-day, 7-day, 1-month) that vendors pay to work in the society. These are pass prices, not penalties or fines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="3">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Accounts Heads</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>Bank Accounts</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>The seeded account 'SBI A/c - Society' is set as your society's primary bank account; every non-cash receipt and payment is booked to it, so the payment QR must belong to this bank. If your society banks elsewhere, change the primary bank account after setup (Settings &gt; Accounts). Do not change default account IDs unless strictly necessary.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="3">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="14" ht="13.8" customHeight="1" s="3">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Brought Forward</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Past Balances</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Ensure brought forward balances from the previous financial year are exact. This is critical for balance sheets.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="3">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="15" ht="13.8" customHeight="1" s="3">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Check before you submit</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Check every step. When you submit, the server creates the society's signing keys and your agreement is generated. After setup, flats' undivided-interest shares are worked out from their areas unless you enter the figures from your Declaration; they must add up to 100% before voting by undivided interest or billing on it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Agreement</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Legal Agreement</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Review the final agreement terms carefully before printing and signing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="3">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Society Details</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>State / Jurisdiction</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>EstateHub is jurisdiction-aware: select the society's state accurately. It decides inter-state (IGST) vs intra-state (CGST+SGST) tax on RCM vendor payments, and which state's statutory Balance Sheet head-mapping and Sinking/Repair Fund rate defaults apply (jurisdiction-aware rules are fully live for Uttar Pradesh; other states use generic/Union-law figures until their own regime is added).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="3">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Bye-Laws Adoption</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Provisional until a resolution</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Tick what your Association has actually adopted from the Model Bye-Laws 2011. Nothing here changes how dues, voting or NOC work until a General Body resolution (2/3) is recorded by your society admin under Settings &gt; Society governance; it then activates automatically. Clauses the engine enforces (bye-laws 7, 39, 46, 49) can be varied but not dropped. Leave a clause alone if you have not discussed it — it follows the Model Bye-Laws as written.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="13.8" customHeight="1" s="3"/>
-    <row r="15" ht="13.8" customHeight="1" s="3"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Review the agreement carefully. It is signed in the app by your President and Secretary, each confirming with their own login password; once sealed it cannot be edited, and anyone can check a printed copy on the verification page.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>